<commit_message>
bug fixed and implemented new artifacts
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/__enums__.xlsx
+++ b/LubanConfig/DataTables/Datas/__enums__.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\601\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487F7D31-16F9-4E1E-80BB-82E1617243FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76292C3F-9D74-4F53-9FBF-2E0C6D1AB621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>##var</t>
   </si>
@@ -176,6 +176,34 @@
   </si>
   <si>
     <t>GoldIncrease</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallSizeChange</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallSpeedChange</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>ExtraGold</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>BallCritChange</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DeathZone</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>GoldChange</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>MonsterSpawn</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -194,6 +222,7 @@
     <font>
       <sz val="9"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -294,13 +323,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -578,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -614,13 +643,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -800,7 +829,7 @@
       </c>
     </row>
     <row r="18" spans="8:10" x14ac:dyDescent="0.2">
-      <c r="H18" s="6" t="s">
+      <c r="H18" s="5" t="s">
         <v>34</v>
       </c>
       <c r="J18">
@@ -808,7 +837,7 @@
       </c>
     </row>
     <row r="19" spans="8:10" x14ac:dyDescent="0.2">
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="6" t="s">
         <v>35</v>
       </c>
       <c r="J19">
@@ -816,7 +845,7 @@
       </c>
     </row>
     <row r="20" spans="8:10" x14ac:dyDescent="0.2">
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="6" t="s">
         <v>36</v>
       </c>
       <c r="J20">
@@ -845,6 +874,62 @@
       </c>
       <c r="J23">
         <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H24" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H25" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H26" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J26">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H27" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J27">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H28" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J28">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J29">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H30" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J30">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>